<commit_message>
Laborattor 2 cod + excel
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexandra\Desktop\Facultate_anul_3\Semestrul2\VVSS\Laborator\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47105AC-6F80-4D56-82B2-5723809BF5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B1CE4C-5F0F-40B9-9996-9C7A9BE5CEEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="650" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9324" yWindow="0" windowWidth="13812" windowHeight="13776" tabRatio="650" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -683,17 +683,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -701,17 +710,8 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1039,11 +1039,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10">
       <c r="B2" s="33" t="s">
@@ -1093,10 +1093,10 @@
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="35"/>
+      <c r="E5" s="38"/>
       <c r="H5" s="17" t="s">
         <v>19</v>
       </c>
@@ -1108,19 +1108,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="35"/>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
@@ -1368,11 +1368,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10">
       <c r="B2" s="33" t="s">
@@ -1404,10 +1404,10 @@
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="37"/>
+      <c r="E4" s="39"/>
       <c r="H4" s="17" t="s">
         <v>18</v>
       </c>
@@ -1422,10 +1422,10 @@
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="35"/>
+      <c r="E5" s="38"/>
       <c r="H5" s="17" t="s">
         <v>19</v>
       </c>
@@ -1437,19 +1437,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="35"/>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
@@ -1682,7 +1682,7 @@
     <col min="1" max="1" width="8.88671875" style="6"/>
     <col min="2" max="2" width="12.21875" style="6" customWidth="1"/>
     <col min="3" max="3" width="16.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="25.88671875" style="6" customWidth="1"/>
+    <col min="4" max="4" width="46.33203125" style="6" customWidth="1"/>
     <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
     <col min="6" max="8" width="8.88671875" style="6"/>
     <col min="9" max="9" width="26.77734375" style="6" customWidth="1"/>
@@ -1694,11 +1694,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10">
       <c r="B2" s="33" t="s">
@@ -1730,10 +1730,10 @@
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="34"/>
       <c r="H4" s="17" t="s">
         <v>18</v>
       </c>
@@ -1748,10 +1748,10 @@
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="E5" s="35"/>
+      <c r="E5" s="38"/>
       <c r="H5" s="17" t="s">
         <v>19</v>
       </c>
@@ -1763,19 +1763,19 @@
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="35"/>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
@@ -2097,11 +2097,11 @@
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10">
       <c r="B2" s="33" t="s">
@@ -2133,10 +2133,10 @@
       <c r="C4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="D4" s="34" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="32"/>
+      <c r="E4" s="34"/>
       <c r="H4" s="17" t="s">
         <v>18</v>
       </c>
@@ -2151,10 +2151,10 @@
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="30"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="17" t="s">
         <v>19</v>
       </c>
@@ -2166,10 +2166,10 @@
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="35"/>
       <c r="F6" s="20"/>
     </row>
     <row r="9" spans="1:10">
@@ -2455,11 +2455,11 @@
       <c r="F30" s="2"/>
     </row>
     <row r="32" spans="2:6">
-      <c r="C32" s="38" t="s">
+      <c r="C32" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="31"/>
       <c r="F32" s="18">
         <v>2</v>
       </c>

</xml_diff>